<commit_message>
Some summarization of results
</commit_message>
<xml_diff>
--- a/Results/HV.xlsx
+++ b/Results/HV.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="15">
   <si>
     <t>HyperVolume</t>
   </si>
@@ -55,6 +55,12 @@
   </si>
   <si>
     <t>SBX_DKMU</t>
+  </si>
+  <si>
+    <t>SBX_Polynomial</t>
+  </si>
+  <si>
+    <t>SBX_DKMutaion</t>
   </si>
 </sst>
 </file>
@@ -6801,11 +6807,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="493050768"/>
-        <c:axId val="493045280"/>
+        <c:axId val="383340264"/>
+        <c:axId val="383338696"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="493050768"/>
+        <c:axId val="383340264"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6862,12 +6868,12 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="493045280"/>
+        <c:crossAx val="383338696"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="493045280"/>
+        <c:axId val="383338696"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0.5"/>
@@ -6925,7 +6931,7 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="493050768"/>
+        <c:crossAx val="383340264"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -7722,11 +7728,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="493049984"/>
-        <c:axId val="493047632"/>
+        <c:axId val="383343400"/>
+        <c:axId val="383343792"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="493049984"/>
+        <c:axId val="383343400"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7783,12 +7789,12 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="493047632"/>
+        <c:crossAx val="383343792"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="493047632"/>
+        <c:axId val="383343792"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7845,7 +7851,7 @@
             <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="493049984"/>
+        <c:crossAx val="383343400"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -7859,6 +7865,1037 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
+      <c:layout/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="it-IT"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="it-IT"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="it-IT"/>
+              <a:t>Average Hypervolume</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="it-IT" baseline="0"/>
+              <a:t> value for generations</a:t>
+            </a:r>
+            <a:endParaRPr lang="it-IT"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="it-IT"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet2!$Z$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>SBX_Polynomial</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet2!$A$6:$A$54</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="49"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>29</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>33</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>34</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>36</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>37</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>38</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>39</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>42</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>43</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>44</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>46</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>47</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>49</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>50</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet2!$Z$6:$Z$54</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="49"/>
+                <c:pt idx="0">
+                  <c:v>60.205915250480622</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>64.181521222198654</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>66.859994795054149</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>69.301278735682018</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>71.367896624390639</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>72.898198813150287</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>74.069403239500147</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>75.140818451427606</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>76.168065627339502</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>77.228050997107871</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>77.960111738025788</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>78.805741703197512</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>79.643407670015662</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>80.121314000557277</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>80.578309713840525</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>80.892843231093153</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>81.178989859717831</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>81.477256659053822</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>81.753568485799377</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>81.96710785630178</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>82.116349841363771</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>82.227169059647807</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>82.393424106409753</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>82.498291666942762</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>82.585801238183791</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>82.68586263929248</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>82.750827684210407</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>82.844165995272789</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>82.924074641531405</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>83.00832417891921</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>83.099040924570005</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>83.155317928250582</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>83.5835793532802</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>83.634257411078039</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>84.047774364968703</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>84.095523325846727</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>84.240693292888722</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>84.607293467109272</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>84.688735142420143</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>84.773306307167715</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>84.887410384834567</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>84.975743932235517</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>85.064708531976947</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>85.603711437721046</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>85.683117209214885</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>85.744813910038772</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>85.768254154094762</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>85.853870147542494</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>86.018469089533113</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet2!$AA$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>SBX_DKMutaion</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet2!$A$6:$A$54</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="49"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>29</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>33</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>34</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>36</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>37</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>38</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>39</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>42</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>43</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>44</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>46</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>47</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>49</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>50</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet2!$AA$6:$AA$54</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="49"/>
+                <c:pt idx="0">
+                  <c:v>61.401374745262146</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>64.28816196722542</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>66.267852948289345</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>68.459453072543198</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>70.396029629900767</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>71.576203278169046</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>72.754790143801841</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>74.330234139458227</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>75.525068051931186</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>76.434368400130253</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>77.056446153899515</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>77.945348805529036</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>78.449640781949427</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>79.031163613599844</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>79.781127558725743</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>80.197740866282615</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>80.579603744573447</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>80.905809363285073</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>81.195717164844524</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>81.469724635435483</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>81.694418347833619</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>81.88740449403096</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>82.049782813433069</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>82.225991004111648</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>82.460678412297924</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>82.578116895214038</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>82.693206420176494</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>82.805776785037068</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>82.924596924390329</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>83.032011994517717</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>83.110206311722578</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>83.195884684573187</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>83.263253072185563</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>83.313533711123142</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>83.362900959916928</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>83.417330881075856</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>83.593544015821806</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>83.642973749211393</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>83.719377209511535</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>83.762206665591563</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>83.81069129317126</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>84.005402024732291</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>84.133155988585671</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>84.153628214340614</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>84.220914867052414</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>84.247011600570232</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>84.293644201560966</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>84.460739739771583</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>84.660165954457895</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="121224800"/>
+        <c:axId val="121224016"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="121224800"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="50"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="it-IT"/>
+                  <a:t>Generations</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="it-IT"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="it-IT"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="121224016"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="121224016"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="50"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="it-IT"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="121224800"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="t"/>
       <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
@@ -7967,6 +9004,46 @@
 </file>
 
 <file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -9038,6 +10115,522 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -9100,6 +10693,36 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>276225</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>581025</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>157162</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -19073,24 +20696,24 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:X54"/>
+  <dimension ref="A1:AA56"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -19135,7 +20758,7 @@
       </c>
       <c r="U4" s="4"/>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
         <v>8</v>
       </c>
@@ -19198,8 +20821,14 @@
       </c>
       <c r="V5" s="2"/>
       <c r="W5" s="2"/>
+      <c r="Z5" t="s">
+        <v>13</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>14</v>
+      </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2</v>
       </c>
@@ -19271,8 +20900,16 @@
         <f>(10-(C6+E6+G6+I6+K6+M6+O6+Q6+S6+U6))/10*100</f>
         <v>38.598625254737854</v>
       </c>
+      <c r="Z6">
+        <f>(B6++D6+F6+H6+J6+L6+N6+P6+R6+T6)*100/10</f>
+        <v>60.205915250480622</v>
+      </c>
+      <c r="AA6">
+        <f t="shared" ref="AA6:AA54" si="0">(C6++E6+G6+I6+K6+M6+O6+Q6+S6+U6)*100/10</f>
+        <v>61.401374745262146</v>
+      </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>3</v>
       </c>
@@ -19337,15 +20974,23 @@
         <v>0.64043391870038702</v>
       </c>
       <c r="W7">
-        <f t="shared" ref="W7:X54" si="0">(10-(B7+D7+F7+H7+J7+L7+N7+P7+R7+T7))/10*100</f>
+        <f t="shared" ref="W7:X54" si="1">(10-(B7+D7+F7+H7+J7+L7+N7+P7+R7+T7))/10*100</f>
         <v>35.818478777801353</v>
       </c>
       <c r="X7">
+        <f t="shared" si="1"/>
+        <v>35.711838032774587</v>
+      </c>
+      <c r="Z7">
+        <f t="shared" ref="Z7:Z54" si="2">(B7++D7+F7+H7+J7+L7+N7+P7+R7+T7)*100/10</f>
+        <v>64.181521222198654</v>
+      </c>
+      <c r="AA7">
         <f t="shared" si="0"/>
-        <v>35.711838032774587</v>
+        <v>64.28816196722542</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>4</v>
       </c>
@@ -19410,15 +21055,23 @@
         <v>0.64759302289008502</v>
       </c>
       <c r="W8">
+        <f t="shared" si="1"/>
+        <v>33.140005204945858</v>
+      </c>
+      <c r="X8">
+        <f t="shared" si="1"/>
+        <v>33.732147051710662</v>
+      </c>
+      <c r="Z8">
+        <f t="shared" si="2"/>
+        <v>66.859994795054149</v>
+      </c>
+      <c r="AA8">
         <f t="shared" si="0"/>
-        <v>33.140005204945858</v>
-      </c>
-      <c r="X8">
-        <f t="shared" si="0"/>
-        <v>33.732147051710662</v>
+        <v>66.267852948289345</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>5</v>
       </c>
@@ -19483,15 +21136,23 @@
         <v>0.69731734379876598</v>
       </c>
       <c r="W9">
+        <f t="shared" si="1"/>
+        <v>30.698721264317985</v>
+      </c>
+      <c r="X9">
+        <f t="shared" si="1"/>
+        <v>31.540546927456809</v>
+      </c>
+      <c r="Z9">
+        <f t="shared" si="2"/>
+        <v>69.301278735682018</v>
+      </c>
+      <c r="AA9">
         <f t="shared" si="0"/>
-        <v>30.698721264317985</v>
-      </c>
-      <c r="X9">
-        <f t="shared" si="0"/>
-        <v>31.540546927456809</v>
+        <v>68.459453072543198</v>
       </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>6</v>
       </c>
@@ -19556,15 +21217,23 @@
         <v>0.72210463056087903</v>
       </c>
       <c r="W10">
+        <f t="shared" si="1"/>
+        <v>28.632103375609365</v>
+      </c>
+      <c r="X10">
+        <f t="shared" si="1"/>
+        <v>29.603970370099237</v>
+      </c>
+      <c r="Z10">
+        <f t="shared" si="2"/>
+        <v>71.367896624390639</v>
+      </c>
+      <c r="AA10">
         <f t="shared" si="0"/>
-        <v>28.632103375609365</v>
-      </c>
-      <c r="X10">
-        <f t="shared" si="0"/>
-        <v>29.603970370099237</v>
+        <v>70.396029629900767</v>
       </c>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>7</v>
       </c>
@@ -19629,15 +21298,23 @@
         <v>0.73186964745538796</v>
       </c>
       <c r="W11">
+        <f t="shared" si="1"/>
+        <v>27.101801186849723</v>
+      </c>
+      <c r="X11">
+        <f t="shared" si="1"/>
+        <v>28.423796721830954</v>
+      </c>
+      <c r="Z11">
+        <f t="shared" si="2"/>
+        <v>72.898198813150287</v>
+      </c>
+      <c r="AA11">
         <f t="shared" si="0"/>
-        <v>27.101801186849723</v>
-      </c>
-      <c r="X11">
-        <f t="shared" si="0"/>
-        <v>28.423796721830954</v>
+        <v>71.576203278169046</v>
       </c>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>8</v>
       </c>
@@ -19702,15 +21379,23 @@
         <v>0.73604592218058995</v>
       </c>
       <c r="W12">
+        <f t="shared" si="1"/>
+        <v>25.930596760499853</v>
+      </c>
+      <c r="X12">
+        <f t="shared" si="1"/>
+        <v>27.245209856198173</v>
+      </c>
+      <c r="Z12">
+        <f t="shared" si="2"/>
+        <v>74.069403239500147</v>
+      </c>
+      <c r="AA12">
         <f t="shared" si="0"/>
-        <v>25.930596760499853</v>
-      </c>
-      <c r="X12">
-        <f t="shared" si="0"/>
-        <v>27.245209856198173</v>
+        <v>72.754790143801841</v>
       </c>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>9</v>
       </c>
@@ -19775,15 +21460,23 @@
         <v>0.75575948080139699</v>
       </c>
       <c r="W13">
+        <f t="shared" si="1"/>
+        <v>24.859181548572391</v>
+      </c>
+      <c r="X13">
+        <f t="shared" si="1"/>
+        <v>25.669765860541773</v>
+      </c>
+      <c r="Z13">
+        <f t="shared" si="2"/>
+        <v>75.140818451427606</v>
+      </c>
+      <c r="AA13">
         <f t="shared" si="0"/>
-        <v>24.859181548572391</v>
-      </c>
-      <c r="X13">
-        <f t="shared" si="0"/>
-        <v>25.669765860541773</v>
+        <v>74.330234139458227</v>
       </c>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>10</v>
       </c>
@@ -19848,15 +21541,23 @@
         <v>0.77137480732601305</v>
       </c>
       <c r="W14">
+        <f t="shared" si="1"/>
+        <v>23.831934372660506</v>
+      </c>
+      <c r="X14">
+        <f t="shared" si="1"/>
+        <v>24.474931948068821</v>
+      </c>
+      <c r="Z14">
+        <f t="shared" si="2"/>
+        <v>76.168065627339502</v>
+      </c>
+      <c r="AA14">
         <f t="shared" si="0"/>
-        <v>23.831934372660506</v>
-      </c>
-      <c r="X14">
-        <f t="shared" si="0"/>
-        <v>24.474931948068821</v>
+        <v>75.525068051931186</v>
       </c>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>11</v>
       </c>
@@ -19921,15 +21622,23 @@
         <v>0.77714771074428901</v>
       </c>
       <c r="W15">
+        <f t="shared" si="1"/>
+        <v>22.771949002892136</v>
+      </c>
+      <c r="X15">
+        <f t="shared" si="1"/>
+        <v>23.565631599869743</v>
+      </c>
+      <c r="Z15">
+        <f t="shared" si="2"/>
+        <v>77.228050997107871</v>
+      </c>
+      <c r="AA15">
         <f t="shared" si="0"/>
-        <v>22.771949002892136</v>
-      </c>
-      <c r="X15">
-        <f t="shared" si="0"/>
-        <v>23.565631599869743</v>
+        <v>76.434368400130253</v>
       </c>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>12</v>
       </c>
@@ -19994,15 +21703,23 @@
         <v>0.78264107449099996</v>
       </c>
       <c r="W16">
+        <f t="shared" si="1"/>
+        <v>22.039888261974212</v>
+      </c>
+      <c r="X16">
+        <f t="shared" si="1"/>
+        <v>22.943553846100482</v>
+      </c>
+      <c r="Z16">
+        <f t="shared" si="2"/>
+        <v>77.960111738025788</v>
+      </c>
+      <c r="AA16">
         <f t="shared" si="0"/>
-        <v>22.039888261974212</v>
-      </c>
-      <c r="X16">
-        <f t="shared" si="0"/>
-        <v>22.943553846100482</v>
+        <v>77.056446153899515</v>
       </c>
     </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>13</v>
       </c>
@@ -20067,15 +21784,23 @@
         <v>0.78855265373866601</v>
       </c>
       <c r="W17">
+        <f t="shared" si="1"/>
+        <v>21.194258296802495</v>
+      </c>
+      <c r="X17">
+        <f t="shared" si="1"/>
+        <v>22.054651194470971</v>
+      </c>
+      <c r="Z17">
+        <f t="shared" si="2"/>
+        <v>78.805741703197512</v>
+      </c>
+      <c r="AA17">
         <f t="shared" si="0"/>
-        <v>21.194258296802495</v>
-      </c>
-      <c r="X17">
-        <f t="shared" si="0"/>
-        <v>22.054651194470971</v>
+        <v>77.945348805529036</v>
       </c>
     </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>14</v>
       </c>
@@ -20140,15 +21865,23 @@
         <v>0.79322419252071996</v>
       </c>
       <c r="W18">
+        <f t="shared" si="1"/>
+        <v>20.356592329984338</v>
+      </c>
+      <c r="X18">
+        <f t="shared" si="1"/>
+        <v>21.55035921805057</v>
+      </c>
+      <c r="Z18">
+        <f t="shared" si="2"/>
+        <v>79.643407670015662</v>
+      </c>
+      <c r="AA18">
         <f t="shared" si="0"/>
-        <v>20.356592329984338</v>
-      </c>
-      <c r="X18">
-        <f t="shared" si="0"/>
-        <v>21.55035921805057</v>
+        <v>78.449640781949427</v>
       </c>
     </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>15</v>
       </c>
@@ -20213,15 +21946,23 @@
         <v>0.80082523321533805</v>
       </c>
       <c r="W19">
+        <f t="shared" si="1"/>
+        <v>19.878685999442727</v>
+      </c>
+      <c r="X19">
+        <f t="shared" si="1"/>
+        <v>20.968836386400156</v>
+      </c>
+      <c r="Z19">
+        <f t="shared" si="2"/>
+        <v>80.121314000557277</v>
+      </c>
+      <c r="AA19">
         <f t="shared" si="0"/>
-        <v>19.878685999442727</v>
-      </c>
-      <c r="X19">
-        <f t="shared" si="0"/>
-        <v>20.968836386400156</v>
+        <v>79.031163613599844</v>
       </c>
     </row>
-    <row r="20" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>16</v>
       </c>
@@ -20286,15 +22027,23 @@
         <v>0.80751080620591897</v>
       </c>
       <c r="W20">
+        <f t="shared" si="1"/>
+        <v>19.421690286159485</v>
+      </c>
+      <c r="X20">
+        <f t="shared" si="1"/>
+        <v>20.218872441274254</v>
+      </c>
+      <c r="Z20">
+        <f t="shared" si="2"/>
+        <v>80.578309713840525</v>
+      </c>
+      <c r="AA20">
         <f t="shared" si="0"/>
-        <v>19.421690286159485</v>
-      </c>
-      <c r="X20">
-        <f t="shared" si="0"/>
-        <v>20.218872441274254</v>
+        <v>79.781127558725743</v>
       </c>
     </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>17</v>
       </c>
@@ -20359,15 +22108,23 @@
         <v>0.80971205225816001</v>
       </c>
       <c r="W21">
+        <f t="shared" si="1"/>
+        <v>19.107156768906854</v>
+      </c>
+      <c r="X21">
+        <f t="shared" si="1"/>
+        <v>19.802259133717381</v>
+      </c>
+      <c r="Z21">
+        <f t="shared" si="2"/>
+        <v>80.892843231093153</v>
+      </c>
+      <c r="AA21">
         <f t="shared" si="0"/>
-        <v>19.107156768906854</v>
-      </c>
-      <c r="X21">
-        <f t="shared" si="0"/>
-        <v>19.802259133717381</v>
+        <v>80.197740866282615</v>
       </c>
     </row>
-    <row r="22" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>18</v>
       </c>
@@ -20432,15 +22189,23 @@
         <v>0.81366647511035395</v>
       </c>
       <c r="W22">
+        <f t="shared" si="1"/>
+        <v>18.821010140282173</v>
+      </c>
+      <c r="X22">
+        <f t="shared" si="1"/>
+        <v>19.420396255426553</v>
+      </c>
+      <c r="Z22">
+        <f t="shared" si="2"/>
+        <v>81.178989859717831</v>
+      </c>
+      <c r="AA22">
         <f t="shared" si="0"/>
-        <v>18.821010140282173</v>
-      </c>
-      <c r="X22">
-        <f t="shared" si="0"/>
-        <v>19.420396255426553</v>
+        <v>80.579603744573447</v>
       </c>
     </row>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>19</v>
       </c>
@@ -20505,15 +22270,23 @@
         <v>0.81493520168586298</v>
       </c>
       <c r="W23">
+        <f t="shared" si="1"/>
+        <v>18.522743340946182</v>
+      </c>
+      <c r="X23">
+        <f t="shared" si="1"/>
+        <v>19.094190636714927</v>
+      </c>
+      <c r="Z23">
+        <f t="shared" si="2"/>
+        <v>81.477256659053822</v>
+      </c>
+      <c r="AA23">
         <f t="shared" si="0"/>
-        <v>18.522743340946182</v>
-      </c>
-      <c r="X23">
-        <f t="shared" si="0"/>
-        <v>19.094190636714927</v>
+        <v>80.905809363285073</v>
       </c>
     </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>20</v>
       </c>
@@ -20578,15 +22351,23 @@
         <v>0.81728434372712899</v>
       </c>
       <c r="W24">
+        <f t="shared" si="1"/>
+        <v>18.246431514200623</v>
+      </c>
+      <c r="X24">
+        <f t="shared" si="1"/>
+        <v>18.804282835155472</v>
+      </c>
+      <c r="Z24">
+        <f t="shared" si="2"/>
+        <v>81.753568485799377</v>
+      </c>
+      <c r="AA24">
         <f t="shared" si="0"/>
-        <v>18.246431514200623</v>
-      </c>
-      <c r="X24">
-        <f t="shared" si="0"/>
-        <v>18.804282835155472</v>
+        <v>81.195717164844524</v>
       </c>
     </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>21</v>
       </c>
@@ -20651,15 +22432,23 @@
         <v>0.81916152194382197</v>
       </c>
       <c r="W25">
+        <f t="shared" si="1"/>
+        <v>18.032892143698227</v>
+      </c>
+      <c r="X25">
+        <f t="shared" si="1"/>
+        <v>18.530275364564517</v>
+      </c>
+      <c r="Z25">
+        <f t="shared" si="2"/>
+        <v>81.96710785630178</v>
+      </c>
+      <c r="AA25">
         <f t="shared" si="0"/>
-        <v>18.032892143698227</v>
-      </c>
-      <c r="X25">
-        <f t="shared" si="0"/>
-        <v>18.530275364564517</v>
+        <v>81.469724635435483</v>
       </c>
     </row>
-    <row r="26" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>22</v>
       </c>
@@ -20724,15 +22513,23 @@
         <v>0.82043039052977496</v>
       </c>
       <c r="W26">
+        <f t="shared" si="1"/>
+        <v>17.883650158636222</v>
+      </c>
+      <c r="X26">
+        <f t="shared" si="1"/>
+        <v>18.305581652166385</v>
+      </c>
+      <c r="Z26">
+        <f t="shared" si="2"/>
+        <v>82.116349841363771</v>
+      </c>
+      <c r="AA26">
         <f t="shared" si="0"/>
-        <v>17.883650158636222</v>
-      </c>
-      <c r="X26">
-        <f t="shared" si="0"/>
-        <v>18.305581652166385</v>
+        <v>81.694418347833619</v>
       </c>
     </row>
-    <row r="27" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>23</v>
       </c>
@@ -20797,15 +22594,23 @@
         <v>0.82317385349970995</v>
       </c>
       <c r="W27">
+        <f t="shared" si="1"/>
+        <v>17.772830940352193</v>
+      </c>
+      <c r="X27">
+        <f t="shared" si="1"/>
+        <v>18.112595505969047</v>
+      </c>
+      <c r="Z27">
+        <f t="shared" si="2"/>
+        <v>82.227169059647807</v>
+      </c>
+      <c r="AA27">
         <f t="shared" si="0"/>
-        <v>17.772830940352193</v>
-      </c>
-      <c r="X27">
-        <f t="shared" si="0"/>
-        <v>18.112595505969047</v>
+        <v>81.88740449403096</v>
       </c>
     </row>
-    <row r="28" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>24</v>
       </c>
@@ -20870,15 +22675,23 @@
         <v>0.82422873338359404</v>
       </c>
       <c r="W28">
+        <f t="shared" si="1"/>
+        <v>17.606575893590257</v>
+      </c>
+      <c r="X28">
+        <f t="shared" si="1"/>
+        <v>17.950217186566935</v>
+      </c>
+      <c r="Z28">
+        <f t="shared" si="2"/>
+        <v>82.393424106409753</v>
+      </c>
+      <c r="AA28">
         <f t="shared" si="0"/>
-        <v>17.606575893590257</v>
-      </c>
-      <c r="X28">
-        <f t="shared" si="0"/>
-        <v>17.950217186566935</v>
+        <v>82.049782813433069</v>
       </c>
     </row>
-    <row r="29" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>25</v>
       </c>
@@ -20943,15 +22756,23 @@
         <v>0.82476998252640399</v>
       </c>
       <c r="W29">
+        <f t="shared" si="1"/>
+        <v>17.501708333057238</v>
+      </c>
+      <c r="X29">
+        <f t="shared" si="1"/>
+        <v>17.774008995888355</v>
+      </c>
+      <c r="Z29">
+        <f t="shared" si="2"/>
+        <v>82.498291666942762</v>
+      </c>
+      <c r="AA29">
         <f t="shared" si="0"/>
-        <v>17.501708333057238</v>
-      </c>
-      <c r="X29">
-        <f t="shared" si="0"/>
-        <v>17.774008995888355</v>
+        <v>82.225991004111648</v>
       </c>
     </row>
-    <row r="30" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>26</v>
       </c>
@@ -21016,15 +22837,23 @@
         <v>0.82581886641372004</v>
       </c>
       <c r="W30">
+        <f t="shared" si="1"/>
+        <v>17.41419876181622</v>
+      </c>
+      <c r="X30">
+        <f t="shared" si="1"/>
+        <v>17.539321587702084</v>
+      </c>
+      <c r="Z30">
+        <f t="shared" si="2"/>
+        <v>82.585801238183791</v>
+      </c>
+      <c r="AA30">
         <f t="shared" si="0"/>
-        <v>17.41419876181622</v>
-      </c>
-      <c r="X30">
-        <f t="shared" si="0"/>
-        <v>17.539321587702084</v>
+        <v>82.460678412297924</v>
       </c>
     </row>
-    <row r="31" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>27</v>
       </c>
@@ -21089,15 +22918,23 @@
         <v>0.82741166608442396</v>
       </c>
       <c r="W31">
+        <f t="shared" si="1"/>
+        <v>17.314137360707527</v>
+      </c>
+      <c r="X31">
+        <f t="shared" si="1"/>
+        <v>17.421883104785962</v>
+      </c>
+      <c r="Z31">
+        <f t="shared" si="2"/>
+        <v>82.68586263929248</v>
+      </c>
+      <c r="AA31">
         <f t="shared" si="0"/>
-        <v>17.314137360707527</v>
-      </c>
-      <c r="X31">
-        <f t="shared" si="0"/>
-        <v>17.421883104785962</v>
+        <v>82.578116895214038</v>
       </c>
     </row>
-    <row r="32" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>28</v>
       </c>
@@ -21162,15 +22999,23 @@
         <v>0.82830736803837202</v>
       </c>
       <c r="W32">
+        <f t="shared" si="1"/>
+        <v>17.2491723157896</v>
+      </c>
+      <c r="X32">
+        <f t="shared" si="1"/>
+        <v>17.306793579823516</v>
+      </c>
+      <c r="Z32">
+        <f t="shared" si="2"/>
+        <v>82.750827684210407</v>
+      </c>
+      <c r="AA32">
         <f t="shared" si="0"/>
-        <v>17.2491723157896</v>
-      </c>
-      <c r="X32">
-        <f t="shared" si="0"/>
-        <v>17.306793579823516</v>
+        <v>82.693206420176494</v>
       </c>
     </row>
-    <row r="33" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>29</v>
       </c>
@@ -21235,15 +23080,23 @@
         <v>0.82953311278585196</v>
       </c>
       <c r="W33">
+        <f t="shared" si="1"/>
+        <v>17.155834004727204</v>
+      </c>
+      <c r="X33">
+        <f t="shared" si="1"/>
+        <v>17.194223214962943</v>
+      </c>
+      <c r="Z33">
+        <f t="shared" si="2"/>
+        <v>82.844165995272789</v>
+      </c>
+      <c r="AA33">
         <f t="shared" si="0"/>
-        <v>17.155834004727204</v>
-      </c>
-      <c r="X33">
-        <f t="shared" si="0"/>
-        <v>17.194223214962943</v>
+        <v>82.805776785037068</v>
       </c>
     </row>
-    <row r="34" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>30</v>
       </c>
@@ -21308,15 +23161,23 @@
         <v>0.83000283600118296</v>
       </c>
       <c r="W34">
+        <f t="shared" si="1"/>
+        <v>17.075925358468584</v>
+      </c>
+      <c r="X34">
+        <f t="shared" si="1"/>
+        <v>17.075403075609668</v>
+      </c>
+      <c r="Z34">
+        <f t="shared" si="2"/>
+        <v>82.924074641531405</v>
+      </c>
+      <c r="AA34">
         <f t="shared" si="0"/>
-        <v>17.075925358468584</v>
-      </c>
-      <c r="X34">
-        <f t="shared" si="0"/>
-        <v>17.075403075609668</v>
+        <v>82.924596924390329</v>
       </c>
     </row>
-    <row r="35" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>31</v>
       </c>
@@ -21381,15 +23242,23 @@
         <v>0.83198173577368295</v>
       </c>
       <c r="W35">
+        <f t="shared" si="1"/>
+        <v>16.991675821080783</v>
+      </c>
+      <c r="X35">
+        <f t="shared" si="1"/>
+        <v>16.96798800548228</v>
+      </c>
+      <c r="Z35">
+        <f t="shared" si="2"/>
+        <v>83.00832417891921</v>
+      </c>
+      <c r="AA35">
         <f t="shared" si="0"/>
-        <v>16.991675821080783</v>
-      </c>
-      <c r="X35">
-        <f t="shared" si="0"/>
-        <v>16.96798800548228</v>
+        <v>83.032011994517717</v>
       </c>
     </row>
-    <row r="36" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>32</v>
       </c>
@@ -21454,15 +23323,23 @@
         <v>0.83319816568789895</v>
       </c>
       <c r="W36">
+        <f t="shared" si="1"/>
+        <v>16.900959075429984</v>
+      </c>
+      <c r="X36">
+        <f t="shared" si="1"/>
+        <v>16.889793688277415</v>
+      </c>
+      <c r="Z36">
+        <f t="shared" si="2"/>
+        <v>83.099040924570005</v>
+      </c>
+      <c r="AA36">
         <f t="shared" si="0"/>
-        <v>16.900959075429984</v>
-      </c>
-      <c r="X36">
-        <f t="shared" si="0"/>
-        <v>16.889793688277415</v>
+        <v>83.110206311722578</v>
       </c>
     </row>
-    <row r="37" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>33</v>
       </c>
@@ -21527,15 +23404,23 @@
         <v>0.83449322731149</v>
       </c>
       <c r="W37">
+        <f t="shared" si="1"/>
+        <v>16.844682071749411</v>
+      </c>
+      <c r="X37">
+        <f t="shared" si="1"/>
+        <v>16.804115315426813</v>
+      </c>
+      <c r="Z37">
+        <f t="shared" si="2"/>
+        <v>83.155317928250582</v>
+      </c>
+      <c r="AA37">
         <f t="shared" si="0"/>
-        <v>16.844682071749411</v>
-      </c>
-      <c r="X37">
-        <f t="shared" si="0"/>
-        <v>16.804115315426813</v>
+        <v>83.195884684573187</v>
       </c>
     </row>
-    <row r="38" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>34</v>
       </c>
@@ -21600,15 +23485,23 @@
         <v>0.83506438280209305</v>
       </c>
       <c r="W38">
+        <f t="shared" si="1"/>
+        <v>16.416420646719807</v>
+      </c>
+      <c r="X38">
+        <f t="shared" si="1"/>
+        <v>16.73674692781443</v>
+      </c>
+      <c r="Z38">
+        <f t="shared" si="2"/>
+        <v>83.5835793532802</v>
+      </c>
+      <c r="AA38">
         <f t="shared" si="0"/>
-        <v>16.416420646719807</v>
-      </c>
-      <c r="X38">
-        <f t="shared" si="0"/>
-        <v>16.73674692781443</v>
+        <v>83.263253072185563</v>
       </c>
     </row>
-    <row r="39" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>35</v>
       </c>
@@ -21673,15 +23566,23 @@
         <v>0.83552843085926898</v>
       </c>
       <c r="W39">
+        <f t="shared" si="1"/>
+        <v>16.365742588921961</v>
+      </c>
+      <c r="X39">
+        <f t="shared" si="1"/>
+        <v>16.686466288876858</v>
+      </c>
+      <c r="Z39">
+        <f t="shared" si="2"/>
+        <v>83.634257411078039</v>
+      </c>
+      <c r="AA39">
         <f t="shared" si="0"/>
-        <v>16.365742588921961</v>
-      </c>
-      <c r="X39">
-        <f t="shared" si="0"/>
-        <v>16.686466288876858</v>
+        <v>83.313533711123142</v>
       </c>
     </row>
-    <row r="40" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>36</v>
       </c>
@@ -21746,15 +23647,23 @@
         <v>0.83571449610013004</v>
       </c>
       <c r="W40">
+        <f t="shared" si="1"/>
+        <v>15.952225635031301</v>
+      </c>
+      <c r="X40">
+        <f t="shared" si="1"/>
+        <v>16.637099040083072</v>
+      </c>
+      <c r="Z40">
+        <f t="shared" si="2"/>
+        <v>84.047774364968703</v>
+      </c>
+      <c r="AA40">
         <f t="shared" si="0"/>
-        <v>15.952225635031301</v>
-      </c>
-      <c r="X40">
-        <f t="shared" si="0"/>
-        <v>16.637099040083072</v>
+        <v>83.362900959916928</v>
       </c>
     </row>
-    <row r="41" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>37</v>
       </c>
@@ -21819,15 +23728,23 @@
         <v>0.83629985263523399</v>
       </c>
       <c r="W41">
+        <f t="shared" si="1"/>
+        <v>15.904476674153276</v>
+      </c>
+      <c r="X41">
+        <f t="shared" si="1"/>
+        <v>16.582669118924134</v>
+      </c>
+      <c r="Z41">
+        <f t="shared" si="2"/>
+        <v>84.095523325846727</v>
+      </c>
+      <c r="AA41">
         <f t="shared" si="0"/>
-        <v>15.904476674153276</v>
-      </c>
-      <c r="X41">
-        <f t="shared" si="0"/>
-        <v>16.582669118924134</v>
+        <v>83.417330881075856</v>
       </c>
     </row>
-    <row r="42" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>38</v>
       </c>
@@ -21892,15 +23809,23 @@
         <v>0.83672836126363204</v>
       </c>
       <c r="W42">
+        <f t="shared" si="1"/>
+        <v>15.759306707111289</v>
+      </c>
+      <c r="X42">
+        <f t="shared" si="1"/>
+        <v>16.406455984178194</v>
+      </c>
+      <c r="Z42">
+        <f t="shared" si="2"/>
+        <v>84.240693292888722</v>
+      </c>
+      <c r="AA42">
         <f t="shared" si="0"/>
-        <v>15.759306707111289</v>
-      </c>
-      <c r="X42">
-        <f t="shared" si="0"/>
-        <v>16.406455984178194</v>
+        <v>83.593544015821806</v>
       </c>
     </row>
-    <row r="43" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>39</v>
       </c>
@@ -21965,15 +23890,23 @@
         <v>0.83714077011527999</v>
       </c>
       <c r="W43">
+        <f t="shared" si="1"/>
+        <v>15.392706532890726</v>
+      </c>
+      <c r="X43">
+        <f t="shared" si="1"/>
+        <v>16.3570262507886</v>
+      </c>
+      <c r="Z43">
+        <f t="shared" si="2"/>
+        <v>84.607293467109272</v>
+      </c>
+      <c r="AA43">
         <f t="shared" si="0"/>
-        <v>15.392706532890726</v>
-      </c>
-      <c r="X43">
-        <f t="shared" si="0"/>
-        <v>16.3570262507886</v>
+        <v>83.642973749211393</v>
       </c>
     </row>
-    <row r="44" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>40</v>
       </c>
@@ -22038,15 +23971,23 @@
         <v>0.837315642829214</v>
       </c>
       <c r="W44">
+        <f t="shared" si="1"/>
+        <v>15.311264857579854</v>
+      </c>
+      <c r="X44">
+        <f t="shared" si="1"/>
+        <v>16.280622790488462</v>
+      </c>
+      <c r="Z44">
+        <f t="shared" si="2"/>
+        <v>84.688735142420143</v>
+      </c>
+      <c r="AA44">
         <f t="shared" si="0"/>
-        <v>15.311264857579854</v>
-      </c>
-      <c r="X44">
-        <f t="shared" si="0"/>
-        <v>16.280622790488462</v>
+        <v>83.719377209511535</v>
       </c>
     </row>
-    <row r="45" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>41</v>
       </c>
@@ -22111,15 +24052,23 @@
         <v>0.83765203927525</v>
       </c>
       <c r="W45">
+        <f t="shared" si="1"/>
+        <v>15.226693692832285</v>
+      </c>
+      <c r="X45">
+        <f t="shared" si="1"/>
+        <v>16.237793334408437</v>
+      </c>
+      <c r="Z45">
+        <f t="shared" si="2"/>
+        <v>84.773306307167715</v>
+      </c>
+      <c r="AA45">
         <f t="shared" si="0"/>
-        <v>15.226693692832285</v>
-      </c>
-      <c r="X45">
-        <f t="shared" si="0"/>
-        <v>16.237793334408437</v>
+        <v>83.762206665591563</v>
       </c>
     </row>
-    <row r="46" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>42</v>
       </c>
@@ -22184,15 +24133,23 @@
         <v>0.838129452093197</v>
       </c>
       <c r="W46">
+        <f t="shared" si="1"/>
+        <v>15.112589615165426</v>
+      </c>
+      <c r="X46">
+        <f t="shared" si="1"/>
+        <v>16.18930870682874</v>
+      </c>
+      <c r="Z46">
+        <f t="shared" si="2"/>
+        <v>84.887410384834567</v>
+      </c>
+      <c r="AA46">
         <f t="shared" si="0"/>
-        <v>15.112589615165426</v>
-      </c>
-      <c r="X46">
-        <f t="shared" si="0"/>
-        <v>16.18930870682874</v>
+        <v>83.81069129317126</v>
       </c>
     </row>
-    <row r="47" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>43</v>
       </c>
@@ -22257,15 +24214,23 @@
         <v>0.83847869259503904</v>
       </c>
       <c r="W47">
+        <f t="shared" si="1"/>
+        <v>15.024256067764483</v>
+      </c>
+      <c r="X47">
+        <f t="shared" si="1"/>
+        <v>15.994597975267713</v>
+      </c>
+      <c r="Z47">
+        <f t="shared" si="2"/>
+        <v>84.975743932235517</v>
+      </c>
+      <c r="AA47">
         <f t="shared" si="0"/>
-        <v>15.024256067764483</v>
-      </c>
-      <c r="X47">
-        <f t="shared" si="0"/>
-        <v>15.994597975267713</v>
+        <v>84.005402024732291</v>
       </c>
     </row>
-    <row r="48" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>44</v>
       </c>
@@ -22330,15 +24295,23 @@
         <v>0.83838734832101003</v>
       </c>
       <c r="W48">
+        <f t="shared" si="1"/>
+        <v>14.935291468023044</v>
+      </c>
+      <c r="X48">
+        <f t="shared" si="1"/>
+        <v>15.866844011414329</v>
+      </c>
+      <c r="Z48">
+        <f t="shared" si="2"/>
+        <v>85.064708531976947</v>
+      </c>
+      <c r="AA48">
         <f t="shared" si="0"/>
-        <v>14.935291468023044</v>
-      </c>
-      <c r="X48">
-        <f t="shared" si="0"/>
-        <v>15.866844011414329</v>
+        <v>84.133155988585671</v>
       </c>
     </row>
-    <row r="49" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>45</v>
       </c>
@@ -22403,15 +24376,23 @@
         <v>0.83883609080800003</v>
       </c>
       <c r="W49">
+        <f t="shared" si="1"/>
+        <v>14.396288562278963</v>
+      </c>
+      <c r="X49">
+        <f t="shared" si="1"/>
+        <v>15.846371785659381</v>
+      </c>
+      <c r="Z49">
+        <f t="shared" si="2"/>
+        <v>85.603711437721046</v>
+      </c>
+      <c r="AA49">
         <f t="shared" si="0"/>
-        <v>14.396288562278963</v>
-      </c>
-      <c r="X49">
-        <f t="shared" si="0"/>
-        <v>15.846371785659381</v>
+        <v>84.153628214340614</v>
       </c>
     </row>
-    <row r="50" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>46</v>
       </c>
@@ -22476,15 +24457,23 @@
         <v>0.83899028259342201</v>
       </c>
       <c r="W50">
+        <f t="shared" si="1"/>
+        <v>14.316882790785126</v>
+      </c>
+      <c r="X50">
+        <f t="shared" si="1"/>
+        <v>15.779085132947584</v>
+      </c>
+      <c r="Z50">
+        <f t="shared" si="2"/>
+        <v>85.683117209214885</v>
+      </c>
+      <c r="AA50">
         <f t="shared" si="0"/>
-        <v>14.316882790785126</v>
-      </c>
-      <c r="X50">
-        <f t="shared" si="0"/>
-        <v>15.779085132947584</v>
+        <v>84.220914867052414</v>
       </c>
     </row>
-    <row r="51" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>47</v>
       </c>
@@ -22549,15 +24538,23 @@
         <v>0.83917862526104903</v>
       </c>
       <c r="W51">
+        <f t="shared" si="1"/>
+        <v>14.25518608996123</v>
+      </c>
+      <c r="X51">
+        <f t="shared" si="1"/>
+        <v>15.752988399429757</v>
+      </c>
+      <c r="Z51">
+        <f t="shared" si="2"/>
+        <v>85.744813910038772</v>
+      </c>
+      <c r="AA51">
         <f t="shared" si="0"/>
-        <v>14.25518608996123</v>
-      </c>
-      <c r="X51">
-        <f t="shared" si="0"/>
-        <v>15.752988399429757</v>
+        <v>84.247011600570232</v>
       </c>
     </row>
-    <row r="52" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>48</v>
       </c>
@@ -22622,15 +24619,23 @@
         <v>0.83911968566671702</v>
       </c>
       <c r="W52">
+        <f t="shared" si="1"/>
+        <v>14.23174584590523</v>
+      </c>
+      <c r="X52">
+        <f t="shared" si="1"/>
+        <v>15.706355798439036</v>
+      </c>
+      <c r="Z52">
+        <f t="shared" si="2"/>
+        <v>85.768254154094762</v>
+      </c>
+      <c r="AA52">
         <f t="shared" si="0"/>
-        <v>14.23174584590523</v>
-      </c>
-      <c r="X52">
-        <f t="shared" si="0"/>
-        <v>15.706355798439036</v>
+        <v>84.293644201560966</v>
       </c>
     </row>
-    <row r="53" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>49</v>
       </c>
@@ -22695,15 +24700,23 @@
         <v>0.83934437774862503</v>
       </c>
       <c r="W53">
+        <f t="shared" si="1"/>
+        <v>14.146129852457518</v>
+      </c>
+      <c r="X53">
+        <f t="shared" si="1"/>
+        <v>15.539260260228414</v>
+      </c>
+      <c r="Z53">
+        <f t="shared" si="2"/>
+        <v>85.853870147542494</v>
+      </c>
+      <c r="AA53">
         <f t="shared" si="0"/>
-        <v>14.146129852457518</v>
-      </c>
-      <c r="X53">
-        <f t="shared" si="0"/>
-        <v>15.539260260228414</v>
+        <v>84.460739739771583</v>
       </c>
     </row>
-    <row r="54" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>50</v>
       </c>
@@ -22768,12 +24781,30 @@
         <v>0.83998996775100498</v>
       </c>
       <c r="W54">
+        <f t="shared" si="1"/>
+        <v>13.981530910466891</v>
+      </c>
+      <c r="X54">
+        <f t="shared" si="1"/>
+        <v>15.339834045542098</v>
+      </c>
+      <c r="Z54">
+        <f t="shared" si="2"/>
+        <v>86.018469089533113</v>
+      </c>
+      <c r="AA54">
         <f t="shared" si="0"/>
-        <v>13.981530910466891</v>
-      </c>
-      <c r="X54">
-        <f t="shared" si="0"/>
-        <v>15.339834045542098</v>
+        <v>84.660165954457895</v>
+      </c>
+    </row>
+    <row r="56" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="X56">
+        <f>ABS(W54-X54)</f>
+        <v>1.3583031350752073</v>
+      </c>
+      <c r="AA56">
+        <f>ABS(Z54-AA54)</f>
+        <v>1.3583031350752179</v>
       </c>
     </row>
   </sheetData>

</xml_diff>